<commit_message>
Revert "Squashed commit of the following:"
This reverts commit bd079152d77f766185aed297cc3a44fb82da6cef.
</commit_message>
<xml_diff>
--- a/DataBase/PBIS_TABLE_INFO.xlsx
+++ b/DataBase/PBIS_TABLE_INFO.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="226">
   <si>
     <t>테이블명</t>
   </si>
@@ -483,7 +483,7 @@
     <t>문제 번호</t>
   </si>
   <si>
-    <t>pbNum</t>
+    <t>pb_um</t>
   </si>
   <si>
     <t>플랜 정보가 담긴 테이블</t>
@@ -616,6 +616,12 @@
   </si>
   <si>
     <t>점수 인덱스</t>
+  </si>
+  <si>
+    <t>시험 카테고리(어떤 문제를 풀었는지)</t>
+  </si>
+  <si>
+    <t>ex_cat</t>
   </si>
   <si>
     <t>1과목 점수</t>
@@ -795,7 +801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K218"/>
+  <dimension ref="A1:K219"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -5847,7 +5853,7 @@
         <v>5</v>
       </c>
       <c r="E212" s="6" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>196</v>
@@ -5856,7 +5862,7 @@
         <v>197</v>
       </c>
       <c r="H212" s="9" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I212" s="6" t="s">
         <v>5</v>
@@ -6045,7 +6051,7 @@
         <v>5</v>
       </c>
       <c r="E218" s="6" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>208</v>
@@ -6054,15 +6060,48 @@
         <v>209</v>
       </c>
       <c r="H218" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I218" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J218" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="K218" s="10"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="6">
+        <v>11</v>
+      </c>
+      <c r="B219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F219" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="G219" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H219" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I218" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="J218" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="K218" s="10"/>
+      <c r="I219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J219" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="K219" s="10"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -9086,7 +9125,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -9373,7 +9412,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>196</v>
@@ -9382,7 +9421,7 @@
         <v>197</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>5</v>
@@ -9571,7 +9610,7 @@
         <v>5</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>208</v>
@@ -9580,15 +9619,48 @@
         <v>209</v>
       </c>
       <c r="H18" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="K18" s="10"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6">
+        <v>11</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H19" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="J18" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="K18" s="10"/>
+      <c r="I19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="K19" s="10"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -9791,7 +9863,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M94"/>
+  <dimension ref="A1:M95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -9858,7 +9930,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>21</v>
@@ -9897,7 +9969,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>5</v>
@@ -9936,7 +10008,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>5</v>
@@ -9975,7 +10047,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>5</v>
@@ -10014,7 +10086,7 @@
         <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>21</v>
@@ -10053,7 +10125,7 @@
         <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>5</v>
@@ -10094,7 +10166,7 @@
         <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>5</v>
@@ -10133,7 +10205,7 @@
         <v>43</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>21</v>
@@ -10172,7 +10244,7 @@
         <v>43</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>5</v>
@@ -10213,7 +10285,7 @@
         <v>43</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>5</v>
@@ -10252,7 +10324,7 @@
         <v>43</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>5</v>
@@ -10291,7 +10363,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>21</v>
@@ -10330,7 +10402,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>5</v>
@@ -10371,7 +10443,7 @@
         <v>55</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>5</v>
@@ -10410,7 +10482,7 @@
         <v>55</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>5</v>
@@ -10449,7 +10521,7 @@
         <v>55</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>5</v>
@@ -10488,7 +10560,7 @@
         <v>55</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>5</v>
@@ -10527,7 +10599,7 @@
         <v>55</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>5</v>
@@ -10566,7 +10638,7 @@
         <v>55</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>5</v>
@@ -10605,7 +10677,7 @@
         <v>55</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>5</v>
@@ -10644,7 +10716,7 @@
         <v>75</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>21</v>
@@ -10683,7 +10755,7 @@
         <v>75</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>5</v>
@@ -10722,7 +10794,7 @@
         <v>75</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>5</v>
@@ -10761,7 +10833,7 @@
         <v>75</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>5</v>
@@ -10800,7 +10872,7 @@
         <v>75</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>5</v>
@@ -10839,7 +10911,7 @@
         <v>75</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>5</v>
@@ -10878,7 +10950,7 @@
         <v>75</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>5</v>
@@ -10917,7 +10989,7 @@
         <v>75</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>5</v>
@@ -10956,7 +11028,7 @@
         <v>75</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>5</v>
@@ -10995,7 +11067,7 @@
         <v>75</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>5</v>
@@ -11034,7 +11106,7 @@
         <v>75</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>5</v>
@@ -11073,7 +11145,7 @@
         <v>98</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>21</v>
@@ -11112,7 +11184,7 @@
         <v>98</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>5</v>
@@ -11153,7 +11225,7 @@
         <v>98</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>5</v>
@@ -11194,7 +11266,7 @@
         <v>98</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>5</v>
@@ -11233,7 +11305,7 @@
         <v>98</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>5</v>
@@ -11272,7 +11344,7 @@
         <v>98</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>5</v>
@@ -11311,7 +11383,7 @@
         <v>98</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>5</v>
@@ -11350,7 +11422,7 @@
         <v>98</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>5</v>
@@ -11389,7 +11461,7 @@
         <v>115</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>21</v>
@@ -11428,7 +11500,7 @@
         <v>115</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>5</v>
@@ -11469,7 +11541,7 @@
         <v>115</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>5</v>
@@ -11510,7 +11582,7 @@
         <v>115</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>5</v>
@@ -11549,7 +11621,7 @@
         <v>115</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>5</v>
@@ -11588,7 +11660,7 @@
         <v>115</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>5</v>
@@ -11627,7 +11699,7 @@
         <v>115</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>5</v>
@@ -11666,7 +11738,7 @@
         <v>115</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>5</v>
@@ -11705,7 +11777,7 @@
         <v>115</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>5</v>
@@ -11744,7 +11816,7 @@
         <v>115</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>5</v>
@@ -11783,7 +11855,7 @@
         <v>115</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>5</v>
@@ -11822,7 +11894,7 @@
         <v>115</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>5</v>
@@ -11861,7 +11933,7 @@
         <v>115</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>5</v>
@@ -11900,7 +11972,7 @@
         <v>115</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>5</v>
@@ -11941,7 +12013,7 @@
         <v>142</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>21</v>
@@ -11980,7 +12052,7 @@
         <v>142</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>5</v>
@@ -12021,7 +12093,7 @@
         <v>142</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>5</v>
@@ -12062,7 +12134,7 @@
         <v>142</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>5</v>
@@ -12101,7 +12173,7 @@
         <v>142</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>5</v>
@@ -12140,7 +12212,7 @@
         <v>142</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>5</v>
@@ -12179,7 +12251,7 @@
         <v>152</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>21</v>
@@ -12218,7 +12290,7 @@
         <v>152</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>5</v>
@@ -12259,7 +12331,7 @@
         <v>152</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>5</v>
@@ -12298,7 +12370,7 @@
         <v>152</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>5</v>
@@ -12337,7 +12409,7 @@
         <v>158</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>21</v>
@@ -12376,7 +12448,7 @@
         <v>158</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>5</v>
@@ -12417,7 +12489,7 @@
         <v>158</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>5</v>
@@ -12458,7 +12530,7 @@
         <v>158</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>5</v>
@@ -12497,7 +12569,7 @@
         <v>158</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>5</v>
@@ -12536,7 +12608,7 @@
         <v>158</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>5</v>
@@ -12575,7 +12647,7 @@
         <v>158</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>5</v>
@@ -12614,7 +12686,7 @@
         <v>158</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>5</v>
@@ -12651,7 +12723,7 @@
       </c>
       <c r="B73" s="2"/>
       <c r="C73" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>5</v>
@@ -12688,7 +12760,7 @@
         <v>173</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>21</v>
@@ -12727,7 +12799,7 @@
         <v>173</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>5</v>
@@ -12768,7 +12840,7 @@
         <v>173</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>5</v>
@@ -12807,7 +12879,7 @@
         <v>173</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>5</v>
@@ -12846,7 +12918,7 @@
         <v>178</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>21</v>
@@ -12885,7 +12957,7 @@
         <v>178</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>5</v>
@@ -12924,7 +12996,7 @@
         <v>178</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>5</v>
@@ -12963,7 +13035,7 @@
         <v>178</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>5</v>
@@ -13002,7 +13074,7 @@
         <v>178</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>5</v>
@@ -13041,7 +13113,7 @@
         <v>178</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>5</v>
@@ -13080,7 +13152,7 @@
         <v>178</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>5</v>
@@ -13119,7 +13191,7 @@
         <v>192</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D85" s="2" t="s">
         <v>21</v>
@@ -13158,7 +13230,7 @@
         <v>192</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>5</v>
@@ -13199,7 +13271,7 @@
         <v>192</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D87" s="2" t="s">
         <v>5</v>
@@ -13240,7 +13312,7 @@
         <v>192</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>5</v>
@@ -13252,7 +13324,7 @@
         <v>5</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="H88" s="3" t="s">
         <v>196</v>
@@ -13261,7 +13333,7 @@
         <v>197</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K88" s="2" t="s">
         <v>5</v>
@@ -13279,7 +13351,7 @@
         <v>192</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>5</v>
@@ -13318,7 +13390,7 @@
         <v>192</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>5</v>
@@ -13357,7 +13429,7 @@
         <v>192</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>5</v>
@@ -13396,7 +13468,7 @@
         <v>192</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>5</v>
@@ -13435,7 +13507,7 @@
         <v>192</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>5</v>
@@ -13474,7 +13546,7 @@
         <v>192</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>5</v>
@@ -13486,7 +13558,7 @@
         <v>5</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="H94" s="3" t="s">
         <v>208</v>
@@ -13495,15 +13567,54 @@
         <v>209</v>
       </c>
       <c r="J94" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K94" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L94" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="M94" s="4"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="I95" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="J95" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="K94" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="L94" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="M94" s="4"/>
+      <c r="K95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L95" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="M95" s="4"/>
     </row>
   </sheetData>
   <headerFooter/>

</xml_diff>

<commit_message>
Revert "Merge pull request #10 from Ojanghun/CYJ"
This reverts commit 562b86fa645859d6a7c1319f7b3f294174d824de, reversing
changes made to 6e1285752ffd1592e30c9b148d3b4c1ba17b781a.
</commit_message>
<xml_diff>
--- a/DataBase/PBIS_TABLE_INFO.xlsx
+++ b/DataBase/PBIS_TABLE_INFO.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="226">
   <si>
     <t>테이블명</t>
   </si>
@@ -483,7 +483,7 @@
     <t>문제 번호</t>
   </si>
   <si>
-    <t>pbNum</t>
+    <t>pb_um</t>
   </si>
   <si>
     <t>플랜 정보가 담긴 테이블</t>
@@ -616,6 +616,12 @@
   </si>
   <si>
     <t>점수 인덱스</t>
+  </si>
+  <si>
+    <t>시험 카테고리(어떤 문제를 풀었는지)</t>
+  </si>
+  <si>
+    <t>ex_cat</t>
   </si>
   <si>
     <t>1과목 점수</t>
@@ -795,7 +801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K218"/>
+  <dimension ref="A1:K219"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -5847,7 +5853,7 @@
         <v>5</v>
       </c>
       <c r="E212" s="6" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="F212" s="9" t="s">
         <v>196</v>
@@ -5856,7 +5862,7 @@
         <v>197</v>
       </c>
       <c r="H212" s="9" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I212" s="6" t="s">
         <v>5</v>
@@ -6045,7 +6051,7 @@
         <v>5</v>
       </c>
       <c r="E218" s="6" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="F218" s="9" t="s">
         <v>208</v>
@@ -6054,15 +6060,48 @@
         <v>209</v>
       </c>
       <c r="H218" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I218" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J218" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="K218" s="10"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="6">
+        <v>11</v>
+      </c>
+      <c r="B219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F219" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="G219" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H219" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I218" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="J218" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="K218" s="10"/>
+      <c r="I219" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J219" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="K219" s="10"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -9086,7 +9125,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -9373,7 +9412,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>196</v>
@@ -9382,7 +9421,7 @@
         <v>197</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>5</v>
@@ -9571,7 +9610,7 @@
         <v>5</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>208</v>
@@ -9580,15 +9619,48 @@
         <v>209</v>
       </c>
       <c r="H18" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="K18" s="10"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6">
+        <v>11</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="H19" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="J18" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="K18" s="10"/>
+      <c r="I19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="K19" s="10"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -9791,7 +9863,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M94"/>
+  <dimension ref="A1:M95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -9858,7 +9930,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>21</v>
@@ -9897,7 +9969,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>5</v>
@@ -9936,7 +10008,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>5</v>
@@ -9975,7 +10047,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>5</v>
@@ -10014,7 +10086,7 @@
         <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>21</v>
@@ -10053,7 +10125,7 @@
         <v>34</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>5</v>
@@ -10094,7 +10166,7 @@
         <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>5</v>
@@ -10133,7 +10205,7 @@
         <v>43</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>21</v>
@@ -10172,7 +10244,7 @@
         <v>43</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>5</v>
@@ -10213,7 +10285,7 @@
         <v>43</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>5</v>
@@ -10252,7 +10324,7 @@
         <v>43</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>5</v>
@@ -10291,7 +10363,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>21</v>
@@ -10330,7 +10402,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>5</v>
@@ -10371,7 +10443,7 @@
         <v>55</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>5</v>
@@ -10410,7 +10482,7 @@
         <v>55</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>5</v>
@@ -10449,7 +10521,7 @@
         <v>55</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>5</v>
@@ -10488,7 +10560,7 @@
         <v>55</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>5</v>
@@ -10527,7 +10599,7 @@
         <v>55</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>5</v>
@@ -10566,7 +10638,7 @@
         <v>55</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>5</v>
@@ -10605,7 +10677,7 @@
         <v>55</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>5</v>
@@ -10644,7 +10716,7 @@
         <v>75</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>21</v>
@@ -10683,7 +10755,7 @@
         <v>75</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>5</v>
@@ -10722,7 +10794,7 @@
         <v>75</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>5</v>
@@ -10761,7 +10833,7 @@
         <v>75</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>5</v>
@@ -10800,7 +10872,7 @@
         <v>75</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>5</v>
@@ -10839,7 +10911,7 @@
         <v>75</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>5</v>
@@ -10878,7 +10950,7 @@
         <v>75</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>5</v>
@@ -10917,7 +10989,7 @@
         <v>75</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>5</v>
@@ -10956,7 +11028,7 @@
         <v>75</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>5</v>
@@ -10995,7 +11067,7 @@
         <v>75</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>5</v>
@@ -11034,7 +11106,7 @@
         <v>75</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>5</v>
@@ -11073,7 +11145,7 @@
         <v>98</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>21</v>
@@ -11112,7 +11184,7 @@
         <v>98</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>5</v>
@@ -11153,7 +11225,7 @@
         <v>98</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>5</v>
@@ -11194,7 +11266,7 @@
         <v>98</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>5</v>
@@ -11233,7 +11305,7 @@
         <v>98</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>5</v>
@@ -11272,7 +11344,7 @@
         <v>98</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>5</v>
@@ -11311,7 +11383,7 @@
         <v>98</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>5</v>
@@ -11350,7 +11422,7 @@
         <v>98</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>5</v>
@@ -11389,7 +11461,7 @@
         <v>115</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>21</v>
@@ -11428,7 +11500,7 @@
         <v>115</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>5</v>
@@ -11469,7 +11541,7 @@
         <v>115</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>5</v>
@@ -11510,7 +11582,7 @@
         <v>115</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>5</v>
@@ -11549,7 +11621,7 @@
         <v>115</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>5</v>
@@ -11588,7 +11660,7 @@
         <v>115</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>5</v>
@@ -11627,7 +11699,7 @@
         <v>115</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>5</v>
@@ -11666,7 +11738,7 @@
         <v>115</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>5</v>
@@ -11705,7 +11777,7 @@
         <v>115</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>5</v>
@@ -11744,7 +11816,7 @@
         <v>115</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>5</v>
@@ -11783,7 +11855,7 @@
         <v>115</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>5</v>
@@ -11822,7 +11894,7 @@
         <v>115</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>5</v>
@@ -11861,7 +11933,7 @@
         <v>115</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>5</v>
@@ -11900,7 +11972,7 @@
         <v>115</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>5</v>
@@ -11941,7 +12013,7 @@
         <v>142</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>21</v>
@@ -11980,7 +12052,7 @@
         <v>142</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>5</v>
@@ -12021,7 +12093,7 @@
         <v>142</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>5</v>
@@ -12062,7 +12134,7 @@
         <v>142</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>5</v>
@@ -12101,7 +12173,7 @@
         <v>142</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>5</v>
@@ -12140,7 +12212,7 @@
         <v>142</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>5</v>
@@ -12179,7 +12251,7 @@
         <v>152</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>21</v>
@@ -12218,7 +12290,7 @@
         <v>152</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>5</v>
@@ -12259,7 +12331,7 @@
         <v>152</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>5</v>
@@ -12298,7 +12370,7 @@
         <v>152</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>5</v>
@@ -12337,7 +12409,7 @@
         <v>158</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>21</v>
@@ -12376,7 +12448,7 @@
         <v>158</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>5</v>
@@ -12417,7 +12489,7 @@
         <v>158</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>5</v>
@@ -12458,7 +12530,7 @@
         <v>158</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>5</v>
@@ -12497,7 +12569,7 @@
         <v>158</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>5</v>
@@ -12536,7 +12608,7 @@
         <v>158</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>5</v>
@@ -12575,7 +12647,7 @@
         <v>158</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>5</v>
@@ -12614,7 +12686,7 @@
         <v>158</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>5</v>
@@ -12651,7 +12723,7 @@
       </c>
       <c r="B73" s="2"/>
       <c r="C73" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>5</v>
@@ -12688,7 +12760,7 @@
         <v>173</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>21</v>
@@ -12727,7 +12799,7 @@
         <v>173</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>5</v>
@@ -12768,7 +12840,7 @@
         <v>173</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>5</v>
@@ -12807,7 +12879,7 @@
         <v>173</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>5</v>
@@ -12846,7 +12918,7 @@
         <v>178</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>21</v>
@@ -12885,7 +12957,7 @@
         <v>178</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>5</v>
@@ -12924,7 +12996,7 @@
         <v>178</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>5</v>
@@ -12963,7 +13035,7 @@
         <v>178</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>5</v>
@@ -13002,7 +13074,7 @@
         <v>178</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>5</v>
@@ -13041,7 +13113,7 @@
         <v>178</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>5</v>
@@ -13080,7 +13152,7 @@
         <v>178</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>5</v>
@@ -13119,7 +13191,7 @@
         <v>192</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D85" s="2" t="s">
         <v>21</v>
@@ -13158,7 +13230,7 @@
         <v>192</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>5</v>
@@ -13199,7 +13271,7 @@
         <v>192</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D87" s="2" t="s">
         <v>5</v>
@@ -13240,7 +13312,7 @@
         <v>192</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>5</v>
@@ -13252,7 +13324,7 @@
         <v>5</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="H88" s="3" t="s">
         <v>196</v>
@@ -13261,7 +13333,7 @@
         <v>197</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="K88" s="2" t="s">
         <v>5</v>
@@ -13279,7 +13351,7 @@
         <v>192</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>5</v>
@@ -13318,7 +13390,7 @@
         <v>192</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>5</v>
@@ -13357,7 +13429,7 @@
         <v>192</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>5</v>
@@ -13396,7 +13468,7 @@
         <v>192</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>5</v>
@@ -13435,7 +13507,7 @@
         <v>192</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>5</v>
@@ -13474,7 +13546,7 @@
         <v>192</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>5</v>
@@ -13486,7 +13558,7 @@
         <v>5</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="H94" s="3" t="s">
         <v>208</v>
@@ -13495,15 +13567,54 @@
         <v>209</v>
       </c>
       <c r="J94" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K94" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L94" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="M94" s="4"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="I95" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="J95" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="K94" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="L94" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="M94" s="4"/>
+      <c r="K95" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L95" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="M95" s="4"/>
     </row>
   </sheetData>
   <headerFooter/>

</xml_diff>